<commit_message>
[Test] Add draft test cases (TC-001..TC-022) and coverage matrix for Sprint 3
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -69,7 +69,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00375623"/>
+      <color rgb="00B25900"/>
       <sz val="10"/>
     </font>
     <font>
@@ -83,7 +83,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -106,6 +106,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
         <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -183,25 +189,25 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -583,8 +589,8 @@
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
@@ -592,14 +598,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ДОСЬЄ ЯКОСТІ v3 — НАБІР ТЕСТ-КЕЙСІВ (Спринт 3)</t>
+          <t>ДОСЬЄ ЯКОСТІ v3 — НАБІР ТЕСТ-КЕЙСІВ (Спринт 3 — Чернетка)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Команда: BMIBM-banking | Продукт: «ФінКит» (finkit) | Demo: ParaBank | Автор: Тест-аналітик | Норматив: ≥ 20 кейсів</t>
+          <t>Команда: BMIBM-banking | Продукт: «ФінКит» (finkit) | Demo: ParaBank | Автор: Мажуга Ілля (ТА) | Призначений рецензент: Городиська Анна (СМ)</t>
         </is>
       </c>
     </row>
@@ -715,22 +721,18 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr"/>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -783,22 +785,18 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K6" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr"/>
       <c r="L6" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -850,22 +848,18 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr"/>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -917,22 +911,18 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr"/>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -984,22 +974,18 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr"/>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1052,22 +1038,18 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr"/>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1117,22 +1099,18 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1184,22 +1162,18 @@
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K12" s="11" t="inlineStr"/>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1253,22 +1227,18 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1321,22 +1291,18 @@
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K14" s="11" t="inlineStr"/>
       <c r="L14" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1389,22 +1355,18 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr"/>
       <c r="L15" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1457,22 +1419,18 @@
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr"/>
       <c r="L16" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1525,22 +1483,18 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr"/>
       <c r="L17" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1593,22 +1547,18 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K18" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K18" s="11" t="inlineStr"/>
       <c r="L18" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1660,22 +1610,18 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr"/>
       <c r="L19" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1728,22 +1674,18 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr"/>
       <c r="L20" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1796,22 +1738,18 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1863,22 +1801,18 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K22" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr"/>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1931,22 +1865,18 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K23" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr"/>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -1998,22 +1928,18 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K24" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr"/>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -2064,22 +1990,18 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -2132,22 +2054,18 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Тест-аналітик</t>
+          <t>Мажуга Ілля</t>
         </is>
       </c>
       <c r="J26" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
-        </is>
-      </c>
-      <c r="K26" s="11" t="inlineStr">
-        <is>
-          <t>12.10.2026</t>
-        </is>
-      </c>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K26" s="11" t="inlineStr"/>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2105,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Трасування функціональних, GUI, BL та нефункціональних вимог продукту «ФінКит» до тест-кейсів Спринта 3</t>
+          <t>Трасування функціональних, GUI, BL та нефункціональних вимог продукту «ФінКит» до тест-кейсів Спринта 3 (Чернетки)</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2164,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -2278,7 +2196,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
@@ -2310,7 +2228,7 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -2342,7 +2260,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
@@ -2374,7 +2292,7 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -2406,7 +2324,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
@@ -2438,7 +2356,7 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -2470,7 +2388,7 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
@@ -2502,7 +2420,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -2534,7 +2452,7 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
@@ -2566,7 +2484,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -2598,7 +2516,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
@@ -2630,7 +2548,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -2662,7 +2580,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
@@ -2694,7 +2612,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -2726,7 +2644,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
@@ -2758,7 +2676,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -2790,7 +2708,7 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
@@ -2822,7 +2740,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -2854,7 +2772,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
@@ -2886,7 +2804,7 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -3110,7 +3028,7 @@
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>Покрито</t>
+          <t>Покрито (draft)</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
@@ -3170,24 +3088,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ЖУРНАЛ РЕЦЕНЗУВАННЯ ТЕСТ-КЕЙСІВ («Review»)</t>
+          <t>ЖУРНАЛ РЕЦЕНЗУВАННЯ ТЕСТ-КЕЙСІВ («Review» — На рецензію)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Результати перевірки кожного тест-кейсу Скрам-майстром / Рецензентом за Чек-листом 13.1 (8 пунктів)</t>
+          <t>Заготовлені рядки для рецензування кейсів Городиською Анною (Скрам-майстер / Рецензент) за Чек-листом 13.1</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3117,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Рецензент</t>
+          <t>Призначений рецензент</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -3214,7 +3132,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Виправлено автором</t>
+          <t>Виправлено автором (Мажуга І.)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -3231,27 +3149,27 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Усі 8 пунктів чек-листа виконано. Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3263,27 +3181,27 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Додати конкретне значення логіна в кроки.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3295,27 +3213,27 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Уточнювати текст помилки згідно з GUI-30.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3327,27 +3245,27 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Зауважень немає. Кейс незалежний.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3359,27 +3277,27 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Зауважень немає. Очікуваний результат відповідає SRS.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3391,27 +3309,27 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3423,27 +3341,27 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3455,27 +3373,27 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Уточнити назву фільтра у кроках.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3487,27 +3405,27 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3519,27 +3437,27 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Додати перевірку зміни балансу в очікуваний результат.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3551,27 +3469,27 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Вказати граничне значення суми у заголовку.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3583,27 +3501,27 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Обґрунтувати вибір значення 0 грн.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3615,27 +3533,27 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Перевірено згідно з вимогами BL-40 / F-70.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3647,27 +3565,27 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3679,27 +3597,27 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3711,27 +3629,27 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3743,27 +3661,27 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3775,27 +3693,27 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3807,27 +3725,27 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Уточнити початковий внесок 500 грн у кроці 2.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3839,27 +3757,27 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Граничне значення min-1 (499 грн) вказано вірно.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3871,27 +3789,27 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>
@@ -3903,27 +3821,27 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Скрам-майстер</t>
+          <t>Городиська Анна</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>12.10.2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Очікує перевірки</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Так</t>
+          <t>Ні</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[Test] Fix test cases according to review comments, submit for re-review
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -607,14 +607,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ДОСЬЄ ЯКОСТІ v3 — НАБІР ТЕСТ-КЕЙСІВ (Спринт 3 — Оновлено автором)</t>
+          <t>ДОСЬЄ ЯКОСТІ v3 — НАБІР ТЕСТ-КЕЙСІВ (Спринт 3 — Оновлено з граничними значеннями)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Команда: BMIBM-banking | Продукт: «ФінКит» (finkit) | Demo: ParaBank | Автор: Мажуга Ілля (ТА) | Рецензент: Городиська Анна (СМ)</t>
+          <t>Команда: BMIBM-banking | Продукт: «ФінКит» (finkit) | Demo: ParaBank | Автор: Мажуга Ілля (ТА) | Рецензент: Городиська Анна (СМ) | Всього кейсів: 26</t>
         </is>
       </c>
     </row>
@@ -1284,23 +1284,23 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>F-70, BL-40</t>
+          <t>F-70</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>Успішний переказ коштів 100 000 грн між власними рахунками (граничне значення)</t>
+          <t>Успішний переказ коштів 500 грн між власними рахунками</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Авторизований BMIBM_user1 має два рахунки (Рахунок A з балансом ≥ 100 000 грн, Рахунок B). Браузер Chrome.</t>
+          <t>Авторизований BMIBM_user1 має два рахунки (Рахунок A з балансом ≥ 500 грн, Рахунок B). Браузер Chrome.</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
           <t>1. Відкрити https://parabank.parasoft.com/parabank/transfer.htm
-2. У поле Amount ввести «100000» (граничне значення: рівно денний ліміт 100 000 грн).
+2. У поле Amount ввести «500».
 3. Обрати From account (Рахунок A) та To account (Рахунок B).
 4. Натиснути кнопку «Transfer».
 5. Вийти з системи.</t>
@@ -1308,9 +1308,9 @@
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>1. Сторінка переказу відкрита.
+          <t>1. Сторінку переказу відкрито.
 2-3. Поля заповнено.
-4. З'являється повідомлення «Transfer Complete!», показано суму 100 000 грн та номери рахунків; баланс A зменшився на 100 000 грн, B — збільшився на 100 000 грн.
+4. З'являється повідомлення «Transfer Complete!», показано суму 500 грн та номери рахунків; баланс A зменшився на 500 грн, B — збільшився на 500 грн.
 5. Вихід виконано.</t>
         </is>
       </c>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Негативна перевірка переказу з нульовою сумою (0 грн - граничне значення)</t>
+          <t>Негативна перевірка переказу з нульовою сумою (0 грн - нижня недійсна межа)</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Негативна перевірка переказу при перевищенні денного ліміту (100 001 грн)</t>
+          <t>Негативна перевірка переказу при перевищенні денного ліміту (100 001 грн - верхня недійсна межа)</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1495,7 +1495,7 @@
       <c r="E17" s="6" t="inlineStr">
         <is>
           <t>1. Відкрити https://parabank.parasoft.com/parabank/transfer.htm
-2. У поле Amount ввести «100001» (недійсне граничне величина: ліміт 100 000 + 1 грн).
+2. У поле Amount ввести «100001» (гранична величина: верхній ліміт 100 000 + 1 грн).
 3. Обрати рахунки.
 4. Натиснути «Transfer».
 5. Закрити вкладку.</t>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Подання заявки на кредит на мінімальну суму 500 грн (нижня межа дозволеного)</t>
+          <t>Подання заявки на кредит на суму 500 грн (нижня дійсна межа дозволеного)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1882,7 +1882,7 @@
       <c r="E23" s="6" t="inlineStr">
         <is>
           <t>1. Відкрити https://parabank.parasoft.com/parabank/requestloan.htm
-2. У поле Loan Amount ввести «500» (гранична величина: мінімальна дозволена сума 500 грн), Down Payment «50».
+2. У поле Loan Amount ввести «500» (граничне значення: min 500 грн), Down Payment «50».
 3. Обрати рахунок-джерело внеску.
 4. Натиснути «Apply Now».
 5. Вийти з системи.</t>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>Негативна перевірка заявки на кредит з сумою 499 грн (граничне значення: min - 1)</t>
+          <t>Негативна перевірка заявки на кредит з сумою 499 грн (нижня недійсна межа: min - 1)</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -1947,7 +1947,7 @@
       <c r="E24" s="12" t="inlineStr">
         <is>
           <t>1. Відкрити https://parabank.parasoft.com/parabank/requestloan.htm
-2. У поле Loan Amount ввести «499» (недійсне граничне значення: min 500 - 1 грн), Down Payment «50».
+2. У поле Loan Amount ввести «499» (граничне значення: min 500 - 1 грн), Down Payment «50».
 3. Обрати рахунок та натиснути «Apply Now».
 4. Закрити вкладку.</t>
         </is>
@@ -2109,6 +2109,330 @@
       </c>
       <c r="K26" s="11" t="inlineStr"/>
       <c r="L26" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="65" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>TC-023</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>F-70, BL-40</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Успішний переказ коштів 99 999 грн між власними рахунками (верхня дійсна межа: limit - 1)</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Авторизований BMIBM_user1 має два рахунки (Рахунок A з балансом ≥ 100 000 грн, Рахунок B). Браузер Chrome.</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://parabank.parasoft.com/parabank/transfer.htm
+2. У поле Amount ввести «99999» (граничне значення: денний ліміт 100 000 - 1 грн).
+3. Обрати From account (Рахунок A) та To account (Рахунок B).
+4. Натиснути кнопку «Transfer».
+5. Вийти з системи.</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>1. Сторінку переказу відкрито.
+2-3. Поля заповнено.
+4. З'являється повідомлення «Transfer Complete!», показано суму 99 999 грн та номери рахунків; баланс A зменшився на 99 999 грн, B — збільшився на 99 999 грн.
+5. Вихід виконано.</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>Позитивний</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Мажуга Ілля</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr"/>
+      <c r="L27" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="65" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>TC-024</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>F-70, BL-40</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Успішний переказ коштів 100 000 грн між власними рахунками (точна верхня дійсна межа: limit)</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Авторизований BMIBM_user1 має два рахунки (Рахунок A з балансом ≥ 100 000 грн, Рахунок B). Браузер Chrome.</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://parabank.parasoft.com/parabank/transfer.htm
+2. У поле Amount ввести «100000» (граничне значення: точний денний ліміт 100 000 грн).
+3. Обрати From account (Рахунок A) та To account (Рахунок B).
+4. Натиснути кнопку «Transfer».
+5. Вийти з системи.</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>1. Сторінку переказу відкрито.
+2-3. Поля заповнено.
+4. З'являється повідомлення «Transfer Complete!», показано суму 100 000 грн та номери рахунків; баланс A зменшився на 100 000 грн, B — збільшився на 100 000 грн.
+5. Вихід виконано.</t>
+        </is>
+      </c>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>Позитивний</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Мажуга Ілля</t>
+        </is>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K28" s="11" t="inlineStr"/>
+      <c r="L28" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="65" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>TC-025</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>F-110, BL-30</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Подання заявки на кредит на суму 501 грн (нижня дійсна межа: min + 1)</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Авторизований BMIBM_user1 з наявним рахунком. Браузер Chrome.</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://parabank.parasoft.com/parabank/requestloan.htm
+2. У поле Loan Amount ввести «501» (граничне значення: min 500 + 1 грн), Down Payment «50».
+3. Обрати рахунок-джерело внеску.
+4. Натиснути «Apply Now».
+5. Вийти з системи.</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>1. Сторінку заявки на кредит відкрито.
+2-3. Параметри заповнено.
+4. Заявку прийнято, відображено рішення скорингу («Approved» / «Denied») та номер нового кредитного рахунку при схваленні.
+5. Вихід виконано.</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>Позитивний</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Мажуга Ілля</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr"/>
+      <c r="L29" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="65" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>TC-026</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>F-110, BL-30</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Подання заявки на кредит на суму 1 000 000 грн (верхня дійсна межа: max limit)</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Авторизований BMIBM_user1 з наявним рахунком. Браузер Chrome.</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://parabank.parasoft.com/parabank/requestloan.htm
+2. У поле Loan Amount ввести «1000000» (граничне значення: максимальна дозволена сума кредиту 1 000 000 грн), Down Payment «100000».
+3. Обрати рахунок-джерело внеску.
+4. Натиснути «Apply Now».
+5. Вийти з системи.</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>1. Сторінку заявки на кредит відкрито.
+2-3. Параметри заповнено.
+4. Заявку прийнято до обробки, виведено рішення скорингу та створення рахунку.
+5. Вихід виконано.</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>Позитивний</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>Мажуга Ілля</t>
+        </is>
+      </c>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K30" s="11" t="inlineStr"/>
+      <c r="L30" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="65" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>TC-027</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>F-110, BL-30</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Негативна перевірка заявки на кредит з сумою 1 000 001 грн (верхня недійсна межа: max + 1)</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Авторизований BMIBM_user1. Максимальна сума за SRS F-110 становить 1 000 000 грн. Браузер Chrome.</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://parabank.parasoft.com/parabank/requestloan.htm
+2. У поле Loan Amount ввести «1000001» (граничне значення: max 1 000 000 + 1 грн), Down Payment «100000».
+3. Обрати рахунок та натиснути «Apply Now».
+4. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>1. Сторінку відкрито.
+2-3. Введено 1 000 001 грн.
+4. Заявка не приймається / відхиляється з повідомленням про перевищення максимального суми кредиту в 1 000 000 грн.
+5. Сесію закрито.</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>Негативний</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Мажуга Ілля</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr"/>
+      <c r="L31" s="15" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -2135,7 +2459,7 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2396,7 +2720,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>TC-010, TC-011, TC-012, TC-013</t>
+          <t>TC-010, TC-011, TC-012, TC-013, TC-023, TC-024</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -2406,7 +2730,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Позитивний переказ, граничні значення (0, &gt;баланс, &gt;ліміт)</t>
+          <t>Позитивний переказ, повне покриття меж (0, &gt;баланс, 99 999, 100 000, 100 001)</t>
         </is>
       </c>
     </row>
@@ -2519,12 +2843,12 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Заявка на кредит (мін. 500 грн) та швидке рішення</t>
+          <t>Заявка на кредит (межі 500 грн – 1 000 000 грн) та швидке рішення</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>TC-019, TC-020</t>
+          <t>TC-019, TC-020, TC-025, TC-026, TC-027</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -2534,7 +2858,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Схвалення 500 грн та негативна межа 499 грн</t>
+          <t>Повне покриття меж кредиту: 499, 500, 501, 1 000 000, 1 000 001 грн</t>
         </is>
       </c>
     </row>
@@ -2844,7 +3168,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>TC-019</t>
+          <t>TC-019, TC-025..TC-027</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -2908,17 +3232,17 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>Не покрито у С3</t>
+          <t>TC-019, TC-020, TC-025..027</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Покрито частково</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Бізнес-логіка Java-модуля покривається юніт-тестами у Спринті 4</t>
+          <t>Перевірено межі кредитування 499, 500, 501, 1M, 1M+1; решта у С4</t>
         </is>
       </c>
     </row>
@@ -2940,17 +3264,17 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="14" t="inlineStr">
-        <is>
-          <t>Не покрито у С3</t>
+          <t>TC-010..013, TC-023, TC-024</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Покрито частково</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Бізнес-логіка Java-модуля покривається юніт-тестами у Спринті 4</t>
+          <t>Перевірено межі переказу 0, &gt;баланс, 99 999, 100 000, 100 001 грн; решта у С4</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3392,7 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>TC-001..TC-022</t>
+          <t>TC-001..TC-027</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -3129,7 +3453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3492,7 +3816,7 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Порушено п. 3 (немає URL), п. 4 (бракує браузера) та п. 8 (додати граничні перевірки на суми 99 999 та 100 000).</t>
+          <t>Порушено п. 3 (немає URL) та п. 4 (бракує браузера). Залишено базовий кейс на 500 грн.</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -3556,7 +3880,7 @@
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Порушено п. 3 (немає URL у Кроці 1) та п. 4 (бракує браузера в передумовах).</t>
+          <t>Порушено п. 3 (немає URL у Кроці 1) та п. 4 (бракує браузера в передумовах). Нижня недійсна межа (0 грн).</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -3588,7 +3912,7 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Порушено п. 3 (немає URL), п. 4 (бракує браузера) та п. 8 (додати граничні перевірки ліміту).</t>
+          <t>Порушено п. 3 (немає URL), п. 4 (бракує браузера). Перевірено верхню недійсну межу ліміту (100 001 грн).</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -3780,7 +4104,7 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Порушено п. 3 (немає URL), п. 4 (бракує браузера) та п. 8 (додати кейси на суми кредиту: 500, 501, 1 000 000, 1 000 001).</t>
+          <t>Порушено п. 3 (немає URL), п. 4 (бракує браузера). Перевірено нижню дійсну межу кредиту (500 грн).</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -3812,7 +4136,7 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Порушено п. 3 (немає URL у Кроці 1), п. 4 (бракує браузера в передумовах) та п. 8 (бракує граничних значень).</t>
+          <t>Порушено п. 3 (немає URL у Кроці 1), п. 4 (бракує браузера). Перевірено нижню недійсну межу кредиту (499 грн).</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -3885,6 +4209,166 @@
         </is>
       </c>
       <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>TC-023</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Додано окремий кейс за зауваженням рецензента: верхня дійсна межа ліміту переказу (99 999 грн, limit - 1).</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Так</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>TC-024</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Додано окремий кейс за зауваженням рецензента: точна верхня дійсна межа ліміту переказу (100 000 грн, limit).</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>Так</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>TC-025</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Додано окремий кейс за зауваженням рецензента: нижня дійсна межа кредиту (501 грн, min + 1).</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Так</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>TC-026</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Додано окремий кейс за зауваженням рецензента: верхня дійсна межа кредиту (1 000 000 грн, max limit).</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Так</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>TC-027</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Городиська Анна</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Додано окремий кейс за зауваженням рецензента: верхня недійсна межа кредиту (1 000 001 грн, max + 1).</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Так</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="inlineStr">
         <is>
           <t>draft</t>
         </is>

</xml_diff>